<commit_message>
Implement fixed leave payroll rule
</commit_message>
<xml_diff>
--- a/public/atk_template/Mostra Pagave ATK.xlsx
+++ b/public/atk_template/Mostra Pagave ATK.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
   <si>
     <t>Emri</t>
   </si>
@@ -46,10 +46,31 @@
     <t>Aplikohet Tatimi në Paga</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Jo</t>
+    <t>Arines</t>
+  </si>
+  <si>
+    <t>Ajeti</t>
+  </si>
+  <si>
+    <t>32132131</t>
+  </si>
+  <si>
+    <t>Po</t>
+  </si>
+  <si>
+    <t>Gentian</t>
+  </si>
+  <si>
+    <t>1231540087</t>
+  </si>
+  <si>
+    <t>Fjolla</t>
+  </si>
+  <si>
+    <t>Gashi</t>
+  </si>
+  <si>
+    <t>1176116800</t>
   </si>
 </sst>
 </file>
@@ -426,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -469,19 +490,19 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -490,17 +511,93 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" t="s">
-        <v>12</v>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3">
+        <v>650</v>
+      </c>
+      <c r="E3">
+        <v>32.5</v>
+      </c>
+      <c r="F3">
+        <v>32.5</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" t="s">
+        <v>14</v>
       </c>
     </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4">
+        <v>1100</v>
+      </c>
+      <c r="E4">
+        <v>55</v>
+      </c>
+      <c r="F4">
+        <v>55</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>